<commit_message>
Add FY2023-2025 income statement data for Mistras
</commit_message>
<xml_diff>
--- a/excel/mistras_answer_key.xlsx
+++ b/excel/mistras_answer_key.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rithu\Projects\pe-deal-screening-engine\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rithu\Projects\pe-deal-screening-engine\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{58A5DC3C-32F3-4709-8E8E-13C4376DE2B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6EF3E523-9A70-40DA-8ACB-35FE56300C3D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{86B3820A-0EC3-49A7-AC89-EEF969BD1741}"/>
+    <workbookView xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="12336" activeTab="1" xr2:uid="{86B3820A-0EC3-49A7-AC89-EEF969BD1741}"/>
   </bookViews>
   <sheets>
     <sheet name="Source" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="63">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="83" uniqueCount="66">
   <si>
     <t>Field</t>
   </si>
@@ -229,13 +229,26 @@
   </si>
   <si>
     <t>n/a</t>
+  </si>
+  <si>
+    <t>Revenue</t>
+  </si>
+  <si>
+    <t>Income (loss) from operations</t>
+  </si>
+  <si>
+    <t>Weighted average common shares outstanding: Diluted (in shares)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <numFmts count="2">
+    <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="165" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
+  </numFmts>
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -280,6 +293,13 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -298,16 +318,16 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="43" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -316,15 +336,16 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
-  <cellStyles count="2">
+  <cellStyles count="3">
+    <cellStyle name="Comma" xfId="2" builtinId="3"/>
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
@@ -693,7 +714,7 @@
       <c r="A4" t="s">
         <v>6</v>
       </c>
-      <c r="B4" s="5" t="s">
+      <c r="B4" s="4" t="s">
         <v>21</v>
       </c>
     </row>
@@ -709,7 +730,7 @@
       <c r="A6" t="s">
         <v>16</v>
       </c>
-      <c r="B6" s="6" t="s">
+      <c r="B6" s="5" t="s">
         <v>22</v>
       </c>
     </row>
@@ -717,7 +738,7 @@
       <c r="A7" t="s">
         <v>9</v>
       </c>
-      <c r="B7" s="6" t="s">
+      <c r="B7" s="5" t="s">
         <v>23</v>
       </c>
     </row>
@@ -757,7 +778,7 @@
       <c r="A12" t="s">
         <v>15</v>
       </c>
-      <c r="B12" s="4" t="s">
+      <c r="B12" t="s">
         <v>20</v>
       </c>
     </row>
@@ -777,254 +798,285 @@
     <col min="1" max="1" width="17.77734375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="35.44140625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="15.5546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="6" width="7" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="21" bestFit="1" customWidth="1"/>
+    <col min="4" max="6" width="11.21875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="54.109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A1" s="7" t="s">
+      <c r="A1" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="B1" s="7" t="s">
+      <c r="B1" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="C1" s="7" t="s">
+      <c r="C1" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="D1" s="7" t="s">
+      <c r="D1" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="E1" s="7" t="s">
+      <c r="E1" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="F1" s="7" t="s">
+      <c r="F1" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="G1" s="7" t="s">
+      <c r="G1" s="6" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A2" s="8" t="s">
+      <c r="A2" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="B2" s="8" t="s">
+      <c r="B2" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="C2" s="8" t="s">
+      <c r="C2" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="D2" s="9"/>
-      <c r="E2" s="9"/>
-      <c r="F2" s="9"/>
-      <c r="G2" s="8"/>
+      <c r="D2" s="8">
+        <v>724024</v>
+      </c>
+      <c r="E2" s="8">
+        <v>729640</v>
+      </c>
+      <c r="F2" s="8">
+        <v>705473</v>
+      </c>
+      <c r="G2" s="7" t="s">
+        <v>63</v>
+      </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A3" s="8" t="s">
+      <c r="A3" s="7" t="s">
         <v>34</v>
       </c>
-      <c r="B3" s="8" t="s">
+      <c r="B3" s="7" t="s">
         <v>35</v>
       </c>
-      <c r="C3" s="8" t="s">
+      <c r="C3" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="D3" s="9"/>
-      <c r="E3" s="9"/>
-      <c r="F3" s="9"/>
-      <c r="G3" s="8"/>
+      <c r="D3" s="8">
+        <v>40572</v>
+      </c>
+      <c r="E3" s="8">
+        <v>39826</v>
+      </c>
+      <c r="F3" s="8">
+        <v>-1904</v>
+      </c>
+      <c r="G3" s="7" t="s">
+        <v>64</v>
+      </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A4" s="8" t="s">
+      <c r="A4" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="B4" s="8" t="s">
+      <c r="B4" s="7" t="s">
         <v>37</v>
       </c>
-      <c r="C4" s="8" t="s">
+      <c r="C4" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="D4" s="9"/>
-      <c r="E4" s="9"/>
-      <c r="F4" s="9"/>
-      <c r="G4" s="8"/>
+      <c r="D4" s="8">
+        <v>14643</v>
+      </c>
+      <c r="E4" s="8">
+        <v>17067</v>
+      </c>
+      <c r="F4" s="8">
+        <v>16761</v>
+      </c>
+      <c r="G4" s="7" t="s">
+        <v>37</v>
+      </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A5" s="8" t="s">
+      <c r="A5" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="B5" s="8" t="s">
+      <c r="B5" s="7" t="s">
         <v>39</v>
       </c>
-      <c r="C5" s="8" t="s">
+      <c r="C5" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="D5" s="9"/>
-      <c r="E5" s="9"/>
-      <c r="F5" s="9"/>
-      <c r="G5" s="8"/>
+      <c r="D5" s="8">
+        <v>32058</v>
+      </c>
+      <c r="E5" s="8">
+        <v>31608</v>
+      </c>
+      <c r="F5" s="8">
+        <v>30330</v>
+      </c>
+      <c r="G5" s="7" t="s">
+        <v>65</v>
+      </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A6" s="8" t="s">
+      <c r="A6" s="7" t="s">
         <v>40</v>
       </c>
-      <c r="B6" s="8" t="s">
+      <c r="B6" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="C6" s="8" t="s">
+      <c r="C6" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="D6" s="9"/>
-      <c r="E6" s="9"/>
-      <c r="F6" s="9"/>
-      <c r="G6" s="8"/>
+      <c r="D6" s="8"/>
+      <c r="E6" s="8"/>
+      <c r="F6" s="8"/>
+      <c r="G6" s="7"/>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A7" s="8" t="s">
+      <c r="A7" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="B7" s="8" t="s">
+      <c r="B7" s="7" t="s">
         <v>44</v>
       </c>
-      <c r="C7" s="8" t="s">
+      <c r="C7" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="D7" s="9"/>
-      <c r="E7" s="9"/>
-      <c r="F7" s="9"/>
-      <c r="G7" s="8"/>
+      <c r="D7" s="8"/>
+      <c r="E7" s="8"/>
+      <c r="F7" s="8"/>
+      <c r="G7" s="7"/>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A8" s="8" t="s">
+      <c r="A8" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="B8" s="8" t="s">
+      <c r="B8" s="7" t="s">
         <v>46</v>
       </c>
-      <c r="C8" s="8" t="s">
+      <c r="C8" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="D8" s="9"/>
-      <c r="E8" s="9"/>
-      <c r="F8" s="9"/>
-      <c r="G8" s="8"/>
+      <c r="D8" s="8"/>
+      <c r="E8" s="8"/>
+      <c r="F8" s="8"/>
+      <c r="G8" s="7"/>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A9" s="8" t="s">
+      <c r="A9" s="7" t="s">
         <v>47</v>
       </c>
-      <c r="B9" s="8" t="s">
+      <c r="B9" s="7" t="s">
         <v>48</v>
       </c>
-      <c r="C9" s="8" t="s">
+      <c r="C9" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="D9" s="9"/>
-      <c r="E9" s="9"/>
-      <c r="F9" s="9"/>
-      <c r="G9" s="8"/>
+      <c r="D9" s="8"/>
+      <c r="E9" s="8"/>
+      <c r="F9" s="8"/>
+      <c r="G9" s="7"/>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A10" s="8" t="s">
+      <c r="A10" s="7" t="s">
         <v>49</v>
       </c>
-      <c r="B10" s="8" t="s">
+      <c r="B10" s="7" t="s">
         <v>50</v>
       </c>
-      <c r="C10" s="8" t="s">
+      <c r="C10" s="7" t="s">
         <v>51</v>
       </c>
-      <c r="D10" s="9"/>
-      <c r="E10" s="9"/>
-      <c r="F10" s="11" t="s">
+      <c r="D10" s="8"/>
+      <c r="E10" s="8"/>
+      <c r="F10" s="9" t="s">
         <v>62</v>
       </c>
-      <c r="G10" s="8"/>
+      <c r="G10" s="7"/>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A11" s="8" t="s">
+      <c r="A11" s="7" t="s">
         <v>52</v>
       </c>
-      <c r="B11" s="8" t="s">
+      <c r="B11" s="7" t="s">
         <v>53</v>
       </c>
-      <c r="C11" s="8" t="s">
+      <c r="C11" s="7" t="s">
         <v>51</v>
       </c>
-      <c r="D11" s="9"/>
-      <c r="E11" s="9"/>
-      <c r="F11" s="11" t="s">
+      <c r="D11" s="8"/>
+      <c r="E11" s="8"/>
+      <c r="F11" s="9" t="s">
         <v>62</v>
       </c>
-      <c r="G11" s="8"/>
+      <c r="G11" s="7"/>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A12" s="8" t="s">
+      <c r="A12" s="7" t="s">
         <v>54</v>
       </c>
-      <c r="B12" s="8" t="s">
+      <c r="B12" s="7" t="s">
         <v>55</v>
       </c>
-      <c r="C12" s="8" t="s">
+      <c r="C12" s="7" t="s">
         <v>51</v>
       </c>
-      <c r="D12" s="9"/>
-      <c r="E12" s="9"/>
-      <c r="F12" s="11" t="s">
+      <c r="D12" s="8"/>
+      <c r="E12" s="8"/>
+      <c r="F12" s="9" t="s">
         <v>62</v>
       </c>
-      <c r="G12" s="8"/>
+      <c r="G12" s="7"/>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A13" s="8" t="s">
+      <c r="A13" s="7" t="s">
         <v>56</v>
       </c>
-      <c r="B13" s="8" t="s">
+      <c r="B13" s="7" t="s">
         <v>57</v>
       </c>
-      <c r="C13" s="8" t="s">
+      <c r="C13" s="7" t="s">
         <v>51</v>
       </c>
-      <c r="D13" s="9"/>
-      <c r="E13" s="9"/>
-      <c r="F13" s="11" t="s">
+      <c r="D13" s="8"/>
+      <c r="E13" s="8"/>
+      <c r="F13" s="9" t="s">
         <v>62</v>
       </c>
-      <c r="G13" s="8"/>
+      <c r="G13" s="7"/>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A14" s="8" t="s">
+      <c r="A14" s="7" t="s">
         <v>58</v>
       </c>
-      <c r="B14" s="8" t="s">
+      <c r="B14" s="7" t="s">
         <v>59</v>
       </c>
-      <c r="C14" s="8" t="s">
+      <c r="C14" s="7" t="s">
         <v>51</v>
       </c>
-      <c r="D14" s="9"/>
-      <c r="E14" s="9"/>
-      <c r="F14" s="11" t="s">
+      <c r="D14" s="8"/>
+      <c r="E14" s="8"/>
+      <c r="F14" s="9" t="s">
         <v>62</v>
       </c>
-      <c r="G14" s="8"/>
+      <c r="G14" s="7"/>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A15" s="8" t="s">
+      <c r="A15" s="7" t="s">
         <v>60</v>
       </c>
-      <c r="B15" s="8" t="s">
+      <c r="B15" s="7" t="s">
         <v>61</v>
       </c>
-      <c r="C15" s="8" t="s">
+      <c r="C15" s="7" t="s">
         <v>51</v>
       </c>
-      <c r="D15" s="9"/>
+      <c r="D15" s="8"/>
       <c r="E15" s="10"/>
-      <c r="F15" s="11" t="s">
+      <c r="F15" s="9" t="s">
         <v>62</v>
       </c>
-      <c r="G15" s="4"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Add FY2023-2025 cash flow data for Mistras
</commit_message>
<xml_diff>
--- a/excel/mistras_answer_key.xlsx
+++ b/excel/mistras_answer_key.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rithu\Projects\pe-deal-screening-engine\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6EF3E523-9A70-40DA-8ACB-35FE56300C3D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{71E93E00-6EAB-4A49-9293-4C0727A3ACF7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="12336" activeTab="1" xr2:uid="{86B3820A-0EC3-49A7-AC89-EEF969BD1741}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{86B3820A-0EC3-49A7-AC89-EEF969BD1741}"/>
   </bookViews>
   <sheets>
     <sheet name="Source" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="83" uniqueCount="66">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="87" uniqueCount="70">
   <si>
     <t>Field</t>
   </si>
@@ -238,6 +238,18 @@
   </si>
   <si>
     <t>Weighted average common shares outstanding: Diluted (in shares)</t>
+  </si>
+  <si>
+    <t>No acquisition line; investing section reconciles to total, so 0</t>
+  </si>
+  <si>
+    <t>Net cash provided by operating activities</t>
+  </si>
+  <si>
+    <t>Depreciation and amortization</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   Purchase of property, plant and equipment (excludes purchase of intangible assets 4,518 / 5,084 / 2,795 and finance-lease equipment 10,154 / 9,899 / 7,125)</t>
   </si>
 </sst>
 </file>
@@ -246,7 +258,7 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
     <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="165" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="164" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
   </numFmts>
   <fonts count="7" x14ac:knownFonts="1">
     <font>
@@ -323,7 +335,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="43" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -336,13 +348,16 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="5" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Comma" xfId="2" builtinId="3"/>
@@ -927,10 +942,18 @@
       <c r="C6" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="D6" s="8"/>
-      <c r="E6" s="8"/>
-      <c r="F6" s="8"/>
-      <c r="G6" s="7"/>
+      <c r="D6" s="8">
+        <v>31008</v>
+      </c>
+      <c r="E6" s="8">
+        <v>33010</v>
+      </c>
+      <c r="F6" s="8">
+        <v>34099</v>
+      </c>
+      <c r="G6" s="7" t="s">
+        <v>68</v>
+      </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7" s="7" t="s">
@@ -942,12 +965,20 @@
       <c r="C7" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="D7" s="8"/>
-      <c r="E7" s="8"/>
-      <c r="F7" s="8"/>
-      <c r="G7" s="7"/>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="D7" s="8">
+        <v>32981</v>
+      </c>
+      <c r="E7" s="8">
+        <v>50129</v>
+      </c>
+      <c r="F7" s="8">
+        <v>26748</v>
+      </c>
+      <c r="G7" s="7" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A8" s="7" t="s">
         <v>45</v>
       </c>
@@ -957,10 +988,18 @@
       <c r="C8" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="D8" s="8"/>
-      <c r="E8" s="8"/>
-      <c r="F8" s="8"/>
-      <c r="G8" s="7"/>
+      <c r="D8" s="8">
+        <v>24674</v>
+      </c>
+      <c r="E8" s="8">
+        <v>17902</v>
+      </c>
+      <c r="F8" s="8">
+        <v>20854</v>
+      </c>
+      <c r="G8" s="11" t="s">
+        <v>69</v>
+      </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A9" s="7" t="s">
@@ -972,10 +1011,18 @@
       <c r="C9" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="D9" s="8"/>
-      <c r="E9" s="8"/>
-      <c r="F9" s="8"/>
-      <c r="G9" s="7"/>
+      <c r="D9" s="8">
+        <v>0</v>
+      </c>
+      <c r="E9" s="8">
+        <v>0</v>
+      </c>
+      <c r="F9" s="8">
+        <v>0</v>
+      </c>
+      <c r="G9" t="s">
+        <v>66</v>
+      </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A10" s="7" t="s">

</xml_diff>

<commit_message>
Add FY2024-2025 balance sheet data for Mistras
</commit_message>
<xml_diff>
--- a/excel/mistras_answer_key.xlsx
+++ b/excel/mistras_answer_key.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rithu\Projects\pe-deal-screening-engine\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{71E93E00-6EAB-4A49-9293-4C0727A3ACF7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B7D63CFD-0333-4F9F-9C18-A69946015BFA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{86B3820A-0EC3-49A7-AC89-EEF969BD1741}"/>
+    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" activeTab="1" xr2:uid="{86B3820A-0EC3-49A7-AC89-EEF969BD1741}"/>
   </bookViews>
   <sheets>
     <sheet name="Source" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="87" uniqueCount="70">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="74">
   <si>
     <t>Field</t>
   </si>
@@ -250,6 +250,18 @@
   </si>
   <si>
     <t xml:space="preserve">   Purchase of property, plant and equipment (excludes purchase of intangible assets 4,518 / 5,084 / 2,795 and finance-lease equipment 10,154 / 9,899 / 7,125)</t>
+  </si>
+  <si>
+    <t>Cash and cash equivalents</t>
+  </si>
+  <si>
+    <t>Total Mistras Group, Inc. stakeholders equity</t>
+  </si>
+  <si>
+    <t>Current portion of long-term debt</t>
+  </si>
+  <si>
+    <t>Long-term debt, net of current portion</t>
   </si>
 </sst>
 </file>
@@ -1034,12 +1046,18 @@
       <c r="C10" s="7" t="s">
         <v>51</v>
       </c>
-      <c r="D10" s="8"/>
-      <c r="E10" s="8"/>
+      <c r="D10" s="8">
+        <v>28008</v>
+      </c>
+      <c r="E10" s="8">
+        <v>18317</v>
+      </c>
       <c r="F10" s="9" t="s">
         <v>62</v>
       </c>
-      <c r="G10" s="7"/>
+      <c r="G10" s="7" t="s">
+        <v>70</v>
+      </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A11" s="7" t="s">
@@ -1051,12 +1069,18 @@
       <c r="C11" s="7" t="s">
         <v>51</v>
       </c>
-      <c r="D11" s="8"/>
-      <c r="E11" s="8"/>
+      <c r="D11" s="8">
+        <v>12849</v>
+      </c>
+      <c r="E11" s="8">
+        <v>11591</v>
+      </c>
       <c r="F11" s="9" t="s">
         <v>62</v>
       </c>
-      <c r="G11" s="7"/>
+      <c r="G11" t="s">
+        <v>72</v>
+      </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A12" s="7" t="s">
@@ -1068,12 +1092,18 @@
       <c r="C12" s="7" t="s">
         <v>51</v>
       </c>
-      <c r="D12" s="8"/>
-      <c r="E12" s="8"/>
+      <c r="D12" s="8">
+        <v>165143</v>
+      </c>
+      <c r="E12" s="8">
+        <v>158056</v>
+      </c>
       <c r="F12" s="9" t="s">
         <v>62</v>
       </c>
-      <c r="G12" s="7"/>
+      <c r="G12" t="s">
+        <v>73</v>
+      </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A13" s="7" t="s">
@@ -1085,12 +1115,18 @@
       <c r="C13" s="7" t="s">
         <v>51</v>
       </c>
-      <c r="D13" s="8"/>
-      <c r="E13" s="8"/>
+      <c r="D13" s="8">
+        <v>235104</v>
+      </c>
+      <c r="E13" s="8">
+        <v>198568</v>
+      </c>
       <c r="F13" s="9" t="s">
         <v>62</v>
       </c>
-      <c r="G13" s="7"/>
+      <c r="G13" s="7" t="s">
+        <v>71</v>
+      </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A14" s="7" t="s">
@@ -1102,12 +1138,18 @@
       <c r="C14" s="7" t="s">
         <v>51</v>
       </c>
-      <c r="D14" s="8"/>
-      <c r="E14" s="8"/>
+      <c r="D14" s="8">
+        <v>154673</v>
+      </c>
+      <c r="E14" s="8">
+        <v>127281</v>
+      </c>
       <c r="F14" s="9" t="s">
         <v>62</v>
       </c>
-      <c r="G14" s="7"/>
+      <c r="G14" s="7" t="s">
+        <v>59</v>
+      </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A15" s="7" t="s">
@@ -1119,10 +1161,17 @@
       <c r="C15" s="7" t="s">
         <v>51</v>
       </c>
-      <c r="D15" s="8"/>
-      <c r="E15" s="10"/>
+      <c r="D15" s="8">
+        <v>184829</v>
+      </c>
+      <c r="E15" s="10">
+        <v>181442</v>
+      </c>
       <c r="F15" s="9" t="s">
         <v>62</v>
+      </c>
+      <c r="G15" t="s">
+        <v>61</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add FY2024-2025 balance sheet and finance lease data for Mistras
</commit_message>
<xml_diff>
--- a/excel/mistras_answer_key.xlsx
+++ b/excel/mistras_answer_key.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rithu\Projects\pe-deal-screening-engine\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{36655FCD-84CA-4780-83A2-813280523ECF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F7662CE1-3B8D-4B7B-8DA6-2B3A99897DFE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{86B3820A-0EC3-49A7-AC89-EEF969BD1741}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="74">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="80">
   <si>
     <t>Field</t>
   </si>
@@ -261,7 +261,25 @@
     <t>Long-term debt, net of current portion</t>
   </si>
   <si>
-    <t>Total Mistras Group, Inc. stockeholders equity</t>
+    <t>finance_lease_current</t>
+  </si>
+  <si>
+    <t>Finance lease obligations, current</t>
+  </si>
+  <si>
+    <t>finance_lease_noncurrent</t>
+  </si>
+  <si>
+    <t>Finance lease obligations, non-current</t>
+  </si>
+  <si>
+    <t>Current portion of finance lease obligations</t>
+  </si>
+  <si>
+    <t>Obligations under finance leases, net of current portion</t>
+  </si>
+  <si>
+    <t>Total Mistras Group, Inc. stockholders equity</t>
   </si>
 </sst>
 </file>
@@ -347,7 +365,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="43" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -369,6 +387,9 @@
     <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -819,7 +840,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{17BAFE2E-3FE7-491D-A73E-F0797282A0D5}">
-  <dimension ref="A1:G15"/>
+  <dimension ref="A1:G17"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="17.77734375" bestFit="1" customWidth="1"/>
@@ -1125,7 +1146,7 @@
         <v>62</v>
       </c>
       <c r="G13" s="7" t="s">
-        <v>73</v>
+        <v>79</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.3">
@@ -1172,6 +1193,52 @@
       </c>
       <c r="G15" t="s">
         <v>61</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A16" s="12" t="s">
+        <v>73</v>
+      </c>
+      <c r="B16" s="12" t="s">
+        <v>74</v>
+      </c>
+      <c r="C16" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="D16" s="8">
+        <v>7025</v>
+      </c>
+      <c r="E16" s="10">
+        <v>5317</v>
+      </c>
+      <c r="F16" s="9" t="s">
+        <v>62</v>
+      </c>
+      <c r="G16" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A17" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="B17" t="s">
+        <v>76</v>
+      </c>
+      <c r="C17" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="D17" s="8">
+        <v>17340</v>
+      </c>
+      <c r="E17" s="8">
+        <v>15162</v>
+      </c>
+      <c r="F17" s="9" t="s">
+        <v>62</v>
+      </c>
+      <c r="G17" t="s">
+        <v>78</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add EBITDA, margin, growth, FCF, and CapEx metrics to answer key
</commit_message>
<xml_diff>
--- a/excel/mistras_answer_key.xlsx
+++ b/excel/mistras_answer_key.xlsx
@@ -8,13 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rithu\Projects\pe-deal-screening-engine\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F7662CE1-3B8D-4B7B-8DA6-2B3A99897DFE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2B246FA3-883B-440D-849B-9EC8F22B5685}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{86B3820A-0EC3-49A7-AC89-EEF969BD1741}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{86B3820A-0EC3-49A7-AC89-EEF969BD1741}"/>
   </bookViews>
   <sheets>
     <sheet name="Source" sheetId="1" r:id="rId1"/>
     <sheet name="Raw_Data" sheetId="2" r:id="rId2"/>
+    <sheet name="Calculations" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -40,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="80">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="131" uniqueCount="99">
   <si>
     <t>Field</t>
   </si>
@@ -280,17 +281,75 @@
   </si>
   <si>
     <t>Total Mistras Group, Inc. stockholders equity</t>
+  </si>
+  <si>
+    <t>Assumptions</t>
+  </si>
+  <si>
+    <t>Tax rate (for NOPAT)</t>
+  </si>
+  <si>
+    <t>Include finance leases in debt? (1 = yes, 0 = no)</t>
+  </si>
+  <si>
+    <t>Metric</t>
+  </si>
+  <si>
+    <t>How calculated</t>
+  </si>
+  <si>
+    <t>EBITDA</t>
+  </si>
+  <si>
+    <t>Operating income + D&amp;A</t>
+  </si>
+  <si>
+    <t>$000s</t>
+  </si>
+  <si>
+    <t>EBITDA margin</t>
+  </si>
+  <si>
+    <t>EBITDA / Revenue</t>
+  </si>
+  <si>
+    <t>%</t>
+  </si>
+  <si>
+    <t>Revenue growth (YoY)</t>
+  </si>
+  <si>
+    <t>Revenue / prior-year revenue - 1</t>
+  </si>
+  <si>
+    <t>Free cash flow</t>
+  </si>
+  <si>
+    <t>CFO - CapEx</t>
+  </si>
+  <si>
+    <t>FCF conversion</t>
+  </si>
+  <si>
+    <t>FCF / EBITDA</t>
+  </si>
+  <si>
+    <t>CapEx intensity</t>
+  </si>
+  <si>
+    <t>CapEx / Revenue</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="164" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="178" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="8">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -342,13 +401,24 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF0070C0"/>
+      <name val="Arial Unicode MS"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -360,12 +430,13 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="3">
+  <cellStyleXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="43" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -391,11 +462,16 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="9" fontId="4" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="178" fontId="0" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="178" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
-  <cellStyles count="3">
+  <cellStyles count="4">
     <cellStyle name="Comma" xfId="2" builtinId="3"/>
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Percent" xfId="3" builtinId="5"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -728,13 +804,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{80C0DBDA-0A43-4B62-ACF2-60F209C07FC9}">
   <dimension ref="A1:B12"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
     <col min="2" max="2" width="99.109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -742,7 +818,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2">
       <c r="A2" t="s">
         <v>2</v>
       </c>
@@ -750,7 +826,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2">
       <c r="A3" t="s">
         <v>4</v>
       </c>
@@ -758,7 +834,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:2">
       <c r="A4" t="s">
         <v>6</v>
       </c>
@@ -766,7 +842,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:2">
       <c r="A5" t="s">
         <v>7</v>
       </c>
@@ -774,7 +850,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:2">
       <c r="A6" t="s">
         <v>16</v>
       </c>
@@ -782,7 +858,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:2">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -790,7 +866,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:2">
       <c r="A8" t="s">
         <v>17</v>
       </c>
@@ -798,7 +874,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:2">
       <c r="A9" t="s">
         <v>11</v>
       </c>
@@ -806,7 +882,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:2">
       <c r="A10" t="s">
         <v>12</v>
       </c>
@@ -814,7 +890,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:2">
       <c r="A11" t="s">
         <v>14</v>
       </c>
@@ -822,7 +898,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:2">
       <c r="A12" t="s">
         <v>15</v>
       </c>
@@ -841,7 +917,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{17BAFE2E-3FE7-491D-A73E-F0797282A0D5}">
   <dimension ref="A1:G17"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="17.77734375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="35.44140625" bestFit="1" customWidth="1"/>
@@ -850,7 +926,7 @@
     <col min="7" max="7" width="54.109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7">
       <c r="A1" s="6" t="s">
         <v>24</v>
       </c>
@@ -873,7 +949,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:7">
       <c r="A2" s="7" t="s">
         <v>31</v>
       </c>
@@ -896,7 +972,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:7">
       <c r="A3" s="7" t="s">
         <v>34</v>
       </c>
@@ -919,7 +995,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:7">
       <c r="A4" s="7" t="s">
         <v>36</v>
       </c>
@@ -942,7 +1018,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:7">
       <c r="A5" s="7" t="s">
         <v>38</v>
       </c>
@@ -965,7 +1041,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:7">
       <c r="A6" s="7" t="s">
         <v>40</v>
       </c>
@@ -988,7 +1064,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:7">
       <c r="A7" s="7" t="s">
         <v>43</v>
       </c>
@@ -1011,7 +1087,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="8" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:7" ht="43.2">
       <c r="A8" s="7" t="s">
         <v>45</v>
       </c>
@@ -1034,7 +1110,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:7">
       <c r="A9" s="7" t="s">
         <v>47</v>
       </c>
@@ -1057,7 +1133,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:7">
       <c r="A10" s="7" t="s">
         <v>49</v>
       </c>
@@ -1080,7 +1156,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:7">
       <c r="A11" s="7" t="s">
         <v>52</v>
       </c>
@@ -1103,7 +1179,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:7">
       <c r="A12" s="7" t="s">
         <v>54</v>
       </c>
@@ -1126,7 +1202,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:7">
       <c r="A13" s="7" t="s">
         <v>56</v>
       </c>
@@ -1149,7 +1225,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:7">
       <c r="A14" s="7" t="s">
         <v>58</v>
       </c>
@@ -1172,7 +1248,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:7">
       <c r="A15" s="7" t="s">
         <v>60</v>
       </c>
@@ -1195,7 +1271,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="16" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:7" ht="28.8">
       <c r="A16" s="12" t="s">
         <v>73</v>
       </c>
@@ -1218,7 +1294,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="17" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:7" ht="28.8">
       <c r="A17" s="12" t="s">
         <v>75</v>
       </c>
@@ -1239,6 +1315,200 @@
       </c>
       <c r="G17" t="s">
         <v>78</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3A797A05-44FC-480D-A30B-4B4FB18F111E}">
+  <dimension ref="A1:F11"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
+  <cols>
+    <col min="1" max="1" width="30" customWidth="1"/>
+    <col min="2" max="2" width="15.44140625" customWidth="1"/>
+    <col min="4" max="4" width="22.44140625" customWidth="1"/>
+    <col min="5" max="6" width="12.5546875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6">
+      <c r="A1" s="2" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6">
+      <c r="A2" t="s">
+        <v>81</v>
+      </c>
+      <c r="D2" s="13">
+        <v>0.25</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" ht="28.8">
+      <c r="A3" s="12" t="s">
+        <v>82</v>
+      </c>
+      <c r="D3" s="14">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6">
+      <c r="A5" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="F5" s="1" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" ht="28.8">
+      <c r="A6" t="s">
+        <v>85</v>
+      </c>
+      <c r="B6" s="12" t="s">
+        <v>86</v>
+      </c>
+      <c r="C6" t="s">
+        <v>87</v>
+      </c>
+      <c r="D6">
+        <f>Raw_Data!D3+Raw_Data!D6</f>
+        <v>71580</v>
+      </c>
+      <c r="E6">
+        <f>Raw_Data!E3+Raw_Data!E6</f>
+        <v>72836</v>
+      </c>
+      <c r="F6">
+        <f>Raw_Data!F3+Raw_Data!F6</f>
+        <v>32195</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6">
+      <c r="A7" t="s">
+        <v>88</v>
+      </c>
+      <c r="B7" t="s">
+        <v>89</v>
+      </c>
+      <c r="C7" t="s">
+        <v>90</v>
+      </c>
+      <c r="D7" s="15">
+        <f>D6/Raw_Data!D2</f>
+        <v>9.8864126051070131E-2</v>
+      </c>
+      <c r="E7" s="15">
+        <f>E6/Raw_Data!E2</f>
+        <v>9.9824571021325581E-2</v>
+      </c>
+      <c r="F7" s="15">
+        <f>F6/Raw_Data!F2</f>
+        <v>4.5636048438423581E-2</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" ht="28.8">
+      <c r="A8" t="s">
+        <v>91</v>
+      </c>
+      <c r="B8" s="12" t="s">
+        <v>92</v>
+      </c>
+      <c r="C8" t="s">
+        <v>90</v>
+      </c>
+      <c r="D8" s="15">
+        <f>Raw_Data!D2/Raw_Data!E2-1</f>
+        <v>-7.6969464393399356E-3</v>
+      </c>
+      <c r="E8" s="15">
+        <f>Raw_Data!E2/Raw_Data!F2-1</f>
+        <v>3.4256449219176366E-2</v>
+      </c>
+      <c r="F8" s="16" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6">
+      <c r="A9" t="s">
+        <v>93</v>
+      </c>
+      <c r="B9" t="s">
+        <v>94</v>
+      </c>
+      <c r="C9" t="s">
+        <v>87</v>
+      </c>
+      <c r="D9">
+        <f>Raw_Data!D7-Raw_Data!D8</f>
+        <v>8307</v>
+      </c>
+      <c r="E9">
+        <f>Raw_Data!E7-Raw_Data!E8</f>
+        <v>32227</v>
+      </c>
+      <c r="F9">
+        <f>Raw_Data!F7-Raw_Data!F8</f>
+        <v>5894</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6">
+      <c r="A10" t="s">
+        <v>95</v>
+      </c>
+      <c r="B10" t="s">
+        <v>96</v>
+      </c>
+      <c r="C10" t="s">
+        <v>90</v>
+      </c>
+      <c r="D10" s="15">
+        <f>D9/D6</f>
+        <v>0.11605196982397317</v>
+      </c>
+      <c r="E10" s="15">
+        <f t="shared" ref="E10:F10" si="0">E9/E6</f>
+        <v>0.44245977263990333</v>
+      </c>
+      <c r="F10" s="15">
+        <f t="shared" si="0"/>
+        <v>0.1830719055753999</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6">
+      <c r="A11" t="s">
+        <v>97</v>
+      </c>
+      <c r="B11" t="s">
+        <v>98</v>
+      </c>
+      <c r="C11" t="s">
+        <v>90</v>
+      </c>
+      <c r="D11" s="15">
+        <f>Raw_Data!D8/Raw_Data!D2</f>
+        <v>3.4078980807266054E-2</v>
+      </c>
+      <c r="E11" s="15">
+        <f>Raw_Data!E8/Raw_Data!E2</f>
+        <v>2.453538731429198E-2</v>
+      </c>
+      <c r="F11" s="15">
+        <f>Raw_Data!F8/Raw_Data!F2</f>
+        <v>2.9560309182633495E-2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add net debt, leverage, DSO, and ROIC to answer key
</commit_message>
<xml_diff>
--- a/excel/mistras_answer_key.xlsx
+++ b/excel/mistras_answer_key.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rithu\Projects\pe-deal-screening-engine\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2B246FA3-883B-440D-849B-9EC8F22B5685}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{39E40AFD-E975-4810-AAE1-73872C4B6398}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{86B3820A-0EC3-49A7-AC89-EEF969BD1741}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="131" uniqueCount="99">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="160" uniqueCount="116">
   <si>
     <t>Field</t>
   </si>
@@ -338,16 +338,69 @@
   </si>
   <si>
     <t>CapEx / Revenue</t>
+  </si>
+  <si>
+    <t>Total debt</t>
+  </si>
+  <si>
+    <t>ST debt + LT debt + switch x finance leases</t>
+  </si>
+  <si>
+    <t>Net debt</t>
+  </si>
+  <si>
+    <t>Total debt - Cash</t>
+  </si>
+  <si>
+    <t>Net leverage</t>
+  </si>
+  <si>
+    <t>Net debt / EBITDA</t>
+  </si>
+  <si>
+    <t>x</t>
+  </si>
+  <si>
+    <t>DSO</t>
+  </si>
+  <si>
+    <t>Receivables / Revenue x 365</t>
+  </si>
+  <si>
+    <t>days</t>
+  </si>
+  <si>
+    <t>NOPAT</t>
+  </si>
+  <si>
+    <t>Operating income x (1 - tax rate)</t>
+  </si>
+  <si>
+    <t>Invested capital</t>
+  </si>
+  <si>
+    <t>Total debt + Equity - Cash</t>
+  </si>
+  <si>
+    <t>ROIC</t>
+  </si>
+  <si>
+    <t>NOPAT / Avg. invested capital</t>
+  </si>
+  <si>
+    <t>ROIC ex-goodwill</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="3">
+  <numFmts count="5">
     <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="164" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="178" formatCode="0.0%"/>
+    <numFmt numFmtId="165" formatCode="0.0%"/>
+    <numFmt numFmtId="170" formatCode="0.00&quot;x&quot;"/>
+    <numFmt numFmtId="176" formatCode="0.0"/>
   </numFmts>
   <fonts count="8">
     <font>
@@ -436,7 +489,7 @@
     <xf numFmtId="43" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -464,8 +517,10 @@
     </xf>
     <xf numFmtId="9" fontId="4" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="178" fontId="0" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="178" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="170" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Comma" xfId="2" builtinId="3"/>
@@ -1324,7 +1379,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3A797A05-44FC-480D-A30B-4B4FB18F111E}">
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:F19"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="30" customWidth="1"/>
@@ -1511,6 +1566,169 @@
         <v>2.9560309182633495E-2</v>
       </c>
     </row>
+    <row r="12" spans="1:6" ht="43.2">
+      <c r="A12" t="s">
+        <v>99</v>
+      </c>
+      <c r="B12" s="12" t="s">
+        <v>100</v>
+      </c>
+      <c r="C12" t="s">
+        <v>87</v>
+      </c>
+      <c r="D12">
+        <f>Raw_Data!D11+Raw_Data!D12+$D$3*(Raw_Data!D16+Raw_Data!D17)</f>
+        <v>202357</v>
+      </c>
+      <c r="E12">
+        <f>Raw_Data!E11+Raw_Data!E12+$D$3*(Raw_Data!E16+Raw_Data!E17)</f>
+        <v>190126</v>
+      </c>
+      <c r="F12" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6">
+      <c r="A13" t="s">
+        <v>101</v>
+      </c>
+      <c r="B13" t="s">
+        <v>102</v>
+      </c>
+      <c r="C13" t="s">
+        <v>87</v>
+      </c>
+      <c r="D13">
+        <f>D12-Raw_Data!D10</f>
+        <v>174349</v>
+      </c>
+      <c r="E13">
+        <f>E12-Raw_Data!E10</f>
+        <v>171809</v>
+      </c>
+      <c r="F13" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6">
+      <c r="A14" t="s">
+        <v>103</v>
+      </c>
+      <c r="B14" t="s">
+        <v>104</v>
+      </c>
+      <c r="C14" t="s">
+        <v>105</v>
+      </c>
+      <c r="D14" s="17">
+        <f>D13/D6</f>
+        <v>2.435722268790165</v>
+      </c>
+      <c r="E14" s="17">
+        <f>E13/E6</f>
+        <v>2.358847273326377</v>
+      </c>
+      <c r="F14" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" ht="28.8">
+      <c r="A15" t="s">
+        <v>106</v>
+      </c>
+      <c r="B15" s="12" t="s">
+        <v>107</v>
+      </c>
+      <c r="C15" t="s">
+        <v>108</v>
+      </c>
+      <c r="D15" s="18">
+        <f>Raw_Data!D14/Raw_Data!D2*365</f>
+        <v>77.974825420151817</v>
+      </c>
+      <c r="E15" s="18">
+        <f>Raw_Data!E14/Raw_Data!E2*365</f>
+        <v>63.671899841017492</v>
+      </c>
+      <c r="F15" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" ht="28.8">
+      <c r="A16" t="s">
+        <v>109</v>
+      </c>
+      <c r="B16" s="12" t="s">
+        <v>110</v>
+      </c>
+      <c r="C16" t="s">
+        <v>87</v>
+      </c>
+      <c r="D16">
+        <f>Raw_Data!D3*(1-$D$2)</f>
+        <v>30429</v>
+      </c>
+      <c r="E16">
+        <f>Raw_Data!E3*(1-$D$2)</f>
+        <v>29869.5</v>
+      </c>
+      <c r="F16">
+        <f>Raw_Data!F3*(1-$D$2)</f>
+        <v>-1428</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" ht="28.8">
+      <c r="A17" t="s">
+        <v>111</v>
+      </c>
+      <c r="B17" s="12" t="s">
+        <v>112</v>
+      </c>
+      <c r="C17" t="s">
+        <v>87</v>
+      </c>
+      <c r="D17">
+        <f>D12+Raw_Data!D13-Raw_Data!D10</f>
+        <v>409453</v>
+      </c>
+      <c r="E17">
+        <f>E12+Raw_Data!E13-Raw_Data!E10</f>
+        <v>370377</v>
+      </c>
+      <c r="F17" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" ht="28.8">
+      <c r="A18" t="s">
+        <v>113</v>
+      </c>
+      <c r="B18" s="12" t="s">
+        <v>114</v>
+      </c>
+      <c r="C18" t="s">
+        <v>90</v>
+      </c>
+      <c r="D18" s="15">
+        <f>D16/AVERAGE(D17:E17)</f>
+        <v>7.8040085659695058E-2</v>
+      </c>
+      <c r="E18" t="s">
+        <v>62</v>
+      </c>
+      <c r="F18" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6">
+      <c r="A19" t="s">
+        <v>115</v>
+      </c>
+      <c r="D19" s="15">
+        <f>D16/AVERAGE(D17-Raw_Data!D15,E17-Raw_Data!E15)</f>
+        <v>0.14715675393353789</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Add deal valuation and EV/EBITDA to answer key
</commit_message>
<xml_diff>
--- a/excel/mistras_answer_key.xlsx
+++ b/excel/mistras_answer_key.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rithu\Projects\pe-deal-screening-engine\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8593283E-ABC8-412F-9351-E83CFA9238B2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{70B9F170-789D-4B60-8987-64B3F0628476}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{86B3820A-0EC3-49A7-AC89-EEF969BD1741}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="164" uniqueCount="117">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="183" uniqueCount="131">
   <si>
     <t>Field</t>
   </si>
@@ -392,18 +392,61 @@
   </si>
   <si>
     <t>NOPAT / Avg. invested capital excl. goodwill</t>
+  </si>
+  <si>
+    <t>Valuation at deal price</t>
+  </si>
+  <si>
+    <t>Offer price per share</t>
+  </si>
+  <si>
+    <t>Equity value</t>
+  </si>
+  <si>
+    <t>Enterprise value</t>
+  </si>
+  <si>
+    <t>EV / EBITDA</t>
+  </si>
+  <si>
+    <t>Source: 8-K, Ex. 99.1</t>
+  </si>
+  <si>
+    <t>Price x diluted shares</t>
+  </si>
+  <si>
+    <t>Equity value + Net debt</t>
+  </si>
+  <si>
+    <t>EV / FY2025 EBITDA</t>
+  </si>
+  <si>
+    <t>$</t>
+  </si>
+  <si>
+    <t>Enterprise value (announced)</t>
+  </si>
+  <si>
+    <t>EV / EBITDA (announced)</t>
+  </si>
+  <si>
+    <t>Source: 8-K Ex. 99.1, "approximately $866 million"</t>
+  </si>
+  <si>
+    <t>Announced EV / FY2025 EBITDA</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="5">
+  <numFmts count="6">
     <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="164" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="165" formatCode="0.0%"/>
     <numFmt numFmtId="166" formatCode="0.00&quot;x&quot;"/>
     <numFmt numFmtId="167" formatCode="0.0"/>
+    <numFmt numFmtId="172" formatCode="0.00\ &quot;x&quot;"/>
   </numFmts>
   <fonts count="9">
     <font>
@@ -497,7 +540,7 @@
     <xf numFmtId="43" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -530,6 +573,9 @@
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="172" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Comma" xfId="2" builtinId="3"/>
@@ -1388,11 +1434,11 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3A797A05-44FC-480D-A30B-4B4FB18F111E}">
-  <dimension ref="A1:F19"/>
+  <dimension ref="A1:F27"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="30" customWidth="1"/>
-    <col min="2" max="2" width="15.44140625" customWidth="1"/>
+    <col min="2" max="2" width="19.44140625" customWidth="1"/>
     <col min="4" max="4" width="22.44140625" customWidth="1"/>
     <col min="5" max="6" width="12.5546875" bestFit="1" customWidth="1"/>
   </cols>
@@ -1750,6 +1796,99 @@
         <v>62</v>
       </c>
     </row>
+    <row r="21" spans="1:6">
+      <c r="A21" s="1" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6">
+      <c r="A22" t="s">
+        <v>118</v>
+      </c>
+      <c r="B22" t="s">
+        <v>122</v>
+      </c>
+      <c r="C22" t="s">
+        <v>126</v>
+      </c>
+      <c r="D22" s="20">
+        <v>20.350000000000001</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6">
+      <c r="A23" t="s">
+        <v>119</v>
+      </c>
+      <c r="B23" t="s">
+        <v>123</v>
+      </c>
+      <c r="C23" t="s">
+        <v>87</v>
+      </c>
+      <c r="D23" s="22">
+        <f>D22*Raw_Data!D5</f>
+        <v>652380.30000000005</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6">
+      <c r="A24" t="s">
+        <v>120</v>
+      </c>
+      <c r="B24" t="s">
+        <v>124</v>
+      </c>
+      <c r="C24" t="s">
+        <v>87</v>
+      </c>
+      <c r="D24" s="22">
+        <f>D23+D13</f>
+        <v>826729.3</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6">
+      <c r="A25" t="s">
+        <v>121</v>
+      </c>
+      <c r="B25" t="s">
+        <v>125</v>
+      </c>
+      <c r="C25" t="s">
+        <v>105</v>
+      </c>
+      <c r="D25" s="21">
+        <f>D24/D6</f>
+        <v>11.549724783459068</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" ht="43.2">
+      <c r="A26" t="s">
+        <v>127</v>
+      </c>
+      <c r="B26" s="12" t="s">
+        <v>129</v>
+      </c>
+      <c r="C26" t="s">
+        <v>87</v>
+      </c>
+      <c r="D26" s="20">
+        <v>866000</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" ht="28.8">
+      <c r="A27" t="s">
+        <v>128</v>
+      </c>
+      <c r="B27" s="12" t="s">
+        <v>130</v>
+      </c>
+      <c r="C27" t="s">
+        <v>105</v>
+      </c>
+      <c r="D27" s="17">
+        <f>D26/D6</f>
+        <v>12.098351494830958</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Add Scorecard testing Mistras against Ridgeline mandate
</commit_message>
<xml_diff>
--- a/excel/mistras_answer_key.xlsx
+++ b/excel/mistras_answer_key.xlsx
@@ -8,14 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rithu\Projects\pe-deal-screening-engine\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6A34C17F-4D6C-4A10-BB05-10F8C88E5347}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D2ADEC4-97ED-441E-86E1-E8F211B113A4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{86B3820A-0EC3-49A7-AC89-EEF969BD1741}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{86B3820A-0EC3-49A7-AC89-EEF969BD1741}"/>
   </bookViews>
   <sheets>
     <sheet name="Source" sheetId="1" r:id="rId1"/>
     <sheet name="Raw_Data" sheetId="2" r:id="rId2"/>
     <sheet name="Calculations" sheetId="3" r:id="rId3"/>
+    <sheet name="Scorecard" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -41,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="183" uniqueCount="131">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="204" uniqueCount="148">
   <si>
     <t>Field</t>
   </si>
@@ -434,6 +435,57 @@
   </si>
   <si>
     <t>EV / EBITDA (our estimate)</t>
+  </si>
+  <si>
+    <t>Criterion</t>
+  </si>
+  <si>
+    <t>Min</t>
+  </si>
+  <si>
+    <t>Max</t>
+  </si>
+  <si>
+    <t>Mistras FY2025</t>
+  </si>
+  <si>
+    <t>Result</t>
+  </si>
+  <si>
+    <t>Comment</t>
+  </si>
+  <si>
+    <t>Revenue ($000s)</t>
+  </si>
+  <si>
+    <t>EBITDA ($000s)</t>
+  </si>
+  <si>
+    <t>Net leverage (x)</t>
+  </si>
+  <si>
+    <t>EV/EBITDA, announced (x)</t>
+  </si>
+  <si>
+    <t>Criteria passed</t>
+  </si>
+  <si>
+    <t>YoY used; 3-yr CAGR needs FY2022 revenue (pending)</t>
+  </si>
+  <si>
+    <t>Strict EBITDA; company Adjusted EBITDA would be higher</t>
+  </si>
+  <si>
+    <t>Hurt by receivables build-up and interest/taxes in CFO</t>
+  </si>
+  <si>
+    <t>Excludes intangibles and lease-financed equipment</t>
+  </si>
+  <si>
+    <t>Includes finance leases (switch = 1)</t>
+  </si>
+  <si>
+    <t>Above preferred 10x, below 13x ceiling</t>
   </si>
 </sst>
 </file>
@@ -540,7 +592,7 @@
     <xf numFmtId="43" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -576,6 +628,9 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="9" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Comma" xfId="2" builtinId="3"/>
@@ -1892,4 +1947,207 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F291257D-4353-4162-9CE1-13A38F57D968}">
+  <dimension ref="A1:F11"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
+  <cols>
+    <col min="1" max="1" width="23.5546875" customWidth="1"/>
+    <col min="4" max="4" width="14.6640625" customWidth="1"/>
+    <col min="5" max="5" width="10.77734375" customWidth="1"/>
+    <col min="6" max="6" width="49" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6">
+      <c r="A1" s="1" t="s">
+        <v>131</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>132</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>133</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>134</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>135</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6">
+      <c r="A2" t="s">
+        <v>137</v>
+      </c>
+      <c r="B2" s="23">
+        <v>250000</v>
+      </c>
+      <c r="C2" s="23">
+        <v>1000000</v>
+      </c>
+      <c r="D2">
+        <f>Raw_Data!D2</f>
+        <v>724024</v>
+      </c>
+      <c r="E2" t="str">
+        <f>IF(AND(OR(B2="",D2&gt;=B2),OR(C2="",D2&lt;=C2)),"PASS","FAIL")</f>
+        <v>PASS</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6">
+      <c r="A3" t="s">
+        <v>138</v>
+      </c>
+      <c r="B3" s="23">
+        <v>40000</v>
+      </c>
+      <c r="C3" s="23">
+        <v>100000</v>
+      </c>
+      <c r="D3">
+        <f>Calculations!D6</f>
+        <v>71580</v>
+      </c>
+      <c r="E3" t="str">
+        <f t="shared" ref="E3:E9" si="0">IF(AND(OR(B3="",D3&gt;=B3),OR(C3="",D3&lt;=C3)),"PASS","FAIL")</f>
+        <v>PASS</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6">
+      <c r="A4" t="s">
+        <v>91</v>
+      </c>
+      <c r="B4" s="24">
+        <v>0.05</v>
+      </c>
+      <c r="C4" s="23"/>
+      <c r="D4" s="15">
+        <f>Calculations!D8</f>
+        <v>-7.6969464393399356E-3</v>
+      </c>
+      <c r="E4" t="str">
+        <f t="shared" si="0"/>
+        <v>FAIL</v>
+      </c>
+      <c r="F4" s="25" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6">
+      <c r="A5" t="s">
+        <v>88</v>
+      </c>
+      <c r="B5" s="24">
+        <v>0.12</v>
+      </c>
+      <c r="C5" s="23"/>
+      <c r="D5" s="15">
+        <f>Calculations!D7</f>
+        <v>9.8864126051070131E-2</v>
+      </c>
+      <c r="E5" t="str">
+        <f t="shared" si="0"/>
+        <v>FAIL</v>
+      </c>
+      <c r="F5" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6">
+      <c r="A6" t="s">
+        <v>95</v>
+      </c>
+      <c r="B6" s="24">
+        <v>0.7</v>
+      </c>
+      <c r="C6" s="23"/>
+      <c r="D6" s="15">
+        <f>Calculations!D10</f>
+        <v>0.11605196982397317</v>
+      </c>
+      <c r="E6" t="str">
+        <f t="shared" si="0"/>
+        <v>FAIL</v>
+      </c>
+      <c r="F6" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6">
+      <c r="A7" t="s">
+        <v>97</v>
+      </c>
+      <c r="B7" s="23"/>
+      <c r="C7" s="24">
+        <v>0.03</v>
+      </c>
+      <c r="D7" s="15">
+        <f>Calculations!D11</f>
+        <v>3.4078980807266054E-2</v>
+      </c>
+      <c r="E7" t="str">
+        <f t="shared" si="0"/>
+        <v>FAIL</v>
+      </c>
+      <c r="F7" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6">
+      <c r="A8" t="s">
+        <v>139</v>
+      </c>
+      <c r="B8" s="23"/>
+      <c r="C8" s="23">
+        <v>3</v>
+      </c>
+      <c r="D8" s="17">
+        <f>Calculations!D14</f>
+        <v>2.435722268790165</v>
+      </c>
+      <c r="E8" t="str">
+        <f t="shared" si="0"/>
+        <v>PASS</v>
+      </c>
+      <c r="F8" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6">
+      <c r="A9" t="s">
+        <v>140</v>
+      </c>
+      <c r="B9" s="23"/>
+      <c r="C9" s="23">
+        <v>10</v>
+      </c>
+      <c r="D9" s="17">
+        <f>Calculations!D27</f>
+        <v>12.098351494830958</v>
+      </c>
+      <c r="E9" t="str">
+        <f t="shared" si="0"/>
+        <v>FAIL</v>
+      </c>
+      <c r="F9" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6">
+      <c r="A11" t="s">
+        <v>141</v>
+      </c>
+      <c r="E11" t="str">
+        <f>COUNTIF(E2:E9,"PASS")&amp;" of 8"</f>
+        <v>3 of 8</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add FY2022 revenue and 3-year CAGR to answer key
</commit_message>
<xml_diff>
--- a/excel/mistras_answer_key.xlsx
+++ b/excel/mistras_answer_key.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rithu\Projects\pe-deal-screening-engine\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D2ADEC4-97ED-441E-86E1-E8F211B113A4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CABE7593-68AD-4830-BBFB-1A254C4CACDE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{86B3820A-0EC3-49A7-AC89-EEF969BD1741}"/>
   </bookViews>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="204" uniqueCount="148">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="226" uniqueCount="154">
   <si>
     <t>Field</t>
   </si>
@@ -233,9 +233,6 @@
     <t>n/a</t>
   </si>
   <si>
-    <t>Revenue</t>
-  </si>
-  <si>
     <t>Income (loss) from operations</t>
   </si>
   <si>
@@ -470,9 +467,6 @@
     <t>Criteria passed</t>
   </si>
   <si>
-    <t>YoY used; 3-yr CAGR needs FY2022 revenue (pending)</t>
-  </si>
-  <si>
     <t>Strict EBITDA; company Adjusted EBITDA would be higher</t>
   </si>
   <si>
@@ -486,6 +480,30 @@
   </si>
   <si>
     <t>Above preferred 10x, below 13x ceiling</t>
+  </si>
+  <si>
+    <t>FY2022</t>
+  </si>
+  <si>
+    <t>Revenue,    Revenue (FY2022 from 10-K filed 2025-03-11)</t>
+  </si>
+  <si>
+    <t>Second filing (FY2022 revenue)</t>
+  </si>
+  <si>
+    <t>10-K filed 2025-03-11, Acc.</t>
+  </si>
+  <si>
+    <t>Revenue CAGR (3-yr)</t>
+  </si>
+  <si>
+    <t>(FY2025 rev / FY2022 rev)^(1/3) - 1</t>
+  </si>
+  <si>
+    <t>Revenue growth (3-yr CAGR)</t>
+  </si>
+  <si>
+    <t>FY2022-25 CAGR vs. 5% target</t>
   </si>
 </sst>
 </file>
@@ -592,7 +610,7 @@
     <xf numFmtId="43" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -630,7 +648,6 @@
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="9" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Comma" xfId="2" builtinId="3"/>
@@ -968,10 +985,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{80C0DBDA-0A43-4B62-ACF2-60F209C07FC9}">
-  <dimension ref="A1:B12"/>
+  <dimension ref="A1:B13"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="18" customWidth="1"/>
+    <col min="1" max="1" width="25.44140625" customWidth="1"/>
     <col min="2" max="2" width="99.109375" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1069,6 +1086,14 @@
       </c>
       <c r="B12" t="s">
         <v>20</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2">
+      <c r="A13" t="s">
+        <v>148</v>
+      </c>
+      <c r="B13" t="s">
+        <v>149</v>
       </c>
     </row>
   </sheetData>
@@ -1081,17 +1106,18 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{17BAFE2E-3FE7-491D-A73E-F0797282A0D5}">
-  <dimension ref="A1:G17"/>
+  <dimension ref="A1:H17"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="17.77734375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="35.44140625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="15.5546875" bestFit="1" customWidth="1"/>
     <col min="4" max="6" width="11.21875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="54.109375" customWidth="1"/>
+    <col min="7" max="7" width="11.21875" customWidth="1"/>
+    <col min="8" max="8" width="54.109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7">
+    <row r="1" spans="1:8">
       <c r="A1" s="6" t="s">
         <v>24</v>
       </c>
@@ -1111,10 +1137,13 @@
         <v>29</v>
       </c>
       <c r="G1" s="6" t="s">
+        <v>146</v>
+      </c>
+      <c r="H1" s="6" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="2" spans="1:7">
+    <row r="2" spans="1:8">
       <c r="A2" s="7" t="s">
         <v>31</v>
       </c>
@@ -1133,11 +1162,14 @@
       <c r="F2" s="8">
         <v>705473</v>
       </c>
-      <c r="G2" s="7" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7">
+      <c r="G2" s="8">
+        <v>687373</v>
+      </c>
+      <c r="H2" s="7" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8">
       <c r="A3" s="7" t="s">
         <v>34</v>
       </c>
@@ -1156,11 +1188,14 @@
       <c r="F3" s="8">
         <v>-1904</v>
       </c>
-      <c r="G3" s="7" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7">
+      <c r="G3" s="9" t="s">
+        <v>62</v>
+      </c>
+      <c r="H3" s="7" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8">
       <c r="A4" s="7" t="s">
         <v>36</v>
       </c>
@@ -1179,11 +1214,14 @@
       <c r="F4" s="8">
         <v>16761</v>
       </c>
-      <c r="G4" s="7" t="s">
+      <c r="G4" s="9" t="s">
+        <v>62</v>
+      </c>
+      <c r="H4" s="7" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="5" spans="1:7">
+    <row r="5" spans="1:8">
       <c r="A5" s="7" t="s">
         <v>38</v>
       </c>
@@ -1202,11 +1240,14 @@
       <c r="F5" s="8">
         <v>30330</v>
       </c>
-      <c r="G5" s="7" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7">
+      <c r="G5" s="9" t="s">
+        <v>62</v>
+      </c>
+      <c r="H5" s="7" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8">
       <c r="A6" s="7" t="s">
         <v>40</v>
       </c>
@@ -1225,11 +1266,14 @@
       <c r="F6" s="8">
         <v>34099</v>
       </c>
-      <c r="G6" s="7" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7">
+      <c r="G6" s="9" t="s">
+        <v>62</v>
+      </c>
+      <c r="H6" s="7" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8">
       <c r="A7" s="7" t="s">
         <v>43</v>
       </c>
@@ -1248,11 +1292,14 @@
       <c r="F7" s="8">
         <v>26748</v>
       </c>
-      <c r="G7" s="7" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" ht="43.2">
+      <c r="G7" s="9" t="s">
+        <v>62</v>
+      </c>
+      <c r="H7" s="7" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" ht="43.2">
       <c r="A8" s="7" t="s">
         <v>45</v>
       </c>
@@ -1271,11 +1318,14 @@
       <c r="F8" s="8">
         <v>20854</v>
       </c>
-      <c r="G8" s="11" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7">
+      <c r="G8" s="9" t="s">
+        <v>62</v>
+      </c>
+      <c r="H8" s="11" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8">
       <c r="A9" s="7" t="s">
         <v>47</v>
       </c>
@@ -1294,11 +1344,14 @@
       <c r="F9" s="8">
         <v>0</v>
       </c>
-      <c r="G9" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7">
+      <c r="G9" s="9" t="s">
+        <v>62</v>
+      </c>
+      <c r="H9" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8">
       <c r="A10" s="7" t="s">
         <v>49</v>
       </c>
@@ -1317,11 +1370,14 @@
       <c r="F10" s="9" t="s">
         <v>62</v>
       </c>
-      <c r="G10" s="7" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7">
+      <c r="G10" s="9" t="s">
+        <v>62</v>
+      </c>
+      <c r="H10" s="7" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8">
       <c r="A11" s="7" t="s">
         <v>52</v>
       </c>
@@ -1340,11 +1396,14 @@
       <c r="F11" s="9" t="s">
         <v>62</v>
       </c>
-      <c r="G11" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7">
+      <c r="G11" s="9" t="s">
+        <v>62</v>
+      </c>
+      <c r="H11" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8">
       <c r="A12" s="7" t="s">
         <v>54</v>
       </c>
@@ -1363,11 +1422,14 @@
       <c r="F12" s="9" t="s">
         <v>62</v>
       </c>
-      <c r="G12" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7">
+      <c r="G12" s="9" t="s">
+        <v>62</v>
+      </c>
+      <c r="H12" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8">
       <c r="A13" s="7" t="s">
         <v>56</v>
       </c>
@@ -1386,11 +1448,14 @@
       <c r="F13" s="9" t="s">
         <v>62</v>
       </c>
-      <c r="G13" s="7" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7">
+      <c r="G13" s="9" t="s">
+        <v>62</v>
+      </c>
+      <c r="H13" s="7" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8">
       <c r="A14" s="7" t="s">
         <v>58</v>
       </c>
@@ -1409,11 +1474,14 @@
       <c r="F14" s="9" t="s">
         <v>62</v>
       </c>
-      <c r="G14" s="7" t="s">
+      <c r="G14" s="9" t="s">
+        <v>62</v>
+      </c>
+      <c r="H14" s="7" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="15" spans="1:7">
+    <row r="15" spans="1:8">
       <c r="A15" s="7" t="s">
         <v>60</v>
       </c>
@@ -1432,16 +1500,19 @@
       <c r="F15" s="9" t="s">
         <v>62</v>
       </c>
-      <c r="G15" t="s">
+      <c r="G15" s="9" t="s">
+        <v>62</v>
+      </c>
+      <c r="H15" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="16" spans="1:7" ht="28.8">
+    <row r="16" spans="1:8" ht="28.8">
       <c r="A16" s="12" t="s">
+        <v>72</v>
+      </c>
+      <c r="B16" s="12" t="s">
         <v>73</v>
-      </c>
-      <c r="B16" s="12" t="s">
-        <v>74</v>
       </c>
       <c r="C16" s="7" t="s">
         <v>51</v>
@@ -1455,16 +1526,19 @@
       <c r="F16" s="9" t="s">
         <v>62</v>
       </c>
-      <c r="G16" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="17" spans="1:7" ht="28.8">
+      <c r="G16" s="9" t="s">
+        <v>62</v>
+      </c>
+      <c r="H16" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" ht="28.8">
       <c r="A17" s="12" t="s">
+        <v>74</v>
+      </c>
+      <c r="B17" t="s">
         <v>75</v>
-      </c>
-      <c r="B17" t="s">
-        <v>76</v>
       </c>
       <c r="C17" s="7" t="s">
         <v>51</v>
@@ -1478,8 +1552,11 @@
       <c r="F17" s="9" t="s">
         <v>62</v>
       </c>
-      <c r="G17" t="s">
-        <v>78</v>
+      <c r="G17" s="9" t="s">
+        <v>62</v>
+      </c>
+      <c r="H17" t="s">
+        <v>77</v>
       </c>
     </row>
   </sheetData>
@@ -1500,12 +1577,12 @@
   <sheetData>
     <row r="1" spans="1:6">
       <c r="A1" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="2" spans="1:6">
       <c r="A2" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="D2" s="13">
         <v>0.25</v>
@@ -1513,7 +1590,7 @@
     </row>
     <row r="3" spans="1:6" ht="28.8">
       <c r="A3" s="12" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="D3" s="14">
         <v>1</v>
@@ -1521,10 +1598,10 @@
     </row>
     <row r="5" spans="1:6">
       <c r="A5" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="B5" s="1" t="s">
         <v>83</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>84</v>
       </c>
       <c r="C5" s="1" t="s">
         <v>12</v>
@@ -1541,13 +1618,13 @@
     </row>
     <row r="6" spans="1:6" ht="28.8">
       <c r="A6" t="s">
+        <v>84</v>
+      </c>
+      <c r="B6" s="12" t="s">
         <v>85</v>
       </c>
-      <c r="B6" s="12" t="s">
+      <c r="C6" t="s">
         <v>86</v>
-      </c>
-      <c r="C6" t="s">
-        <v>87</v>
       </c>
       <c r="D6">
         <f>Raw_Data!D3+Raw_Data!D6</f>
@@ -1564,13 +1641,13 @@
     </row>
     <row r="7" spans="1:6">
       <c r="A7" t="s">
+        <v>87</v>
+      </c>
+      <c r="B7" t="s">
         <v>88</v>
       </c>
-      <c r="B7" t="s">
+      <c r="C7" t="s">
         <v>89</v>
-      </c>
-      <c r="C7" t="s">
-        <v>90</v>
       </c>
       <c r="D7" s="15">
         <f>D6/Raw_Data!D2</f>
@@ -1587,13 +1664,13 @@
     </row>
     <row r="8" spans="1:6" ht="28.8">
       <c r="A8" t="s">
+        <v>90</v>
+      </c>
+      <c r="B8" s="12" t="s">
         <v>91</v>
       </c>
-      <c r="B8" s="12" t="s">
-        <v>92</v>
-      </c>
       <c r="C8" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="D8" s="15">
         <f>Raw_Data!D2/Raw_Data!E2-1</f>
@@ -1609,13 +1686,13 @@
     </row>
     <row r="9" spans="1:6">
       <c r="A9" t="s">
+        <v>92</v>
+      </c>
+      <c r="B9" t="s">
         <v>93</v>
       </c>
-      <c r="B9" t="s">
-        <v>94</v>
-      </c>
       <c r="C9" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="D9">
         <f>Raw_Data!D7-Raw_Data!D8</f>
@@ -1632,13 +1709,13 @@
     </row>
     <row r="10" spans="1:6">
       <c r="A10" t="s">
+        <v>94</v>
+      </c>
+      <c r="B10" t="s">
         <v>95</v>
       </c>
-      <c r="B10" t="s">
-        <v>96</v>
-      </c>
       <c r="C10" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="D10" s="15">
         <f>D9/D6</f>
@@ -1655,13 +1732,13 @@
     </row>
     <row r="11" spans="1:6">
       <c r="A11" t="s">
+        <v>96</v>
+      </c>
+      <c r="B11" t="s">
         <v>97</v>
       </c>
-      <c r="B11" t="s">
-        <v>98</v>
-      </c>
       <c r="C11" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="D11" s="15">
         <f>Raw_Data!D8/Raw_Data!D2</f>
@@ -1678,13 +1755,13 @@
     </row>
     <row r="12" spans="1:6" ht="28.8">
       <c r="A12" t="s">
+        <v>98</v>
+      </c>
+      <c r="B12" s="12" t="s">
         <v>99</v>
       </c>
-      <c r="B12" s="12" t="s">
-        <v>100</v>
-      </c>
       <c r="C12" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="D12">
         <f>Raw_Data!D11+Raw_Data!D12+$D$3*(Raw_Data!D16+Raw_Data!D17)</f>
@@ -1700,13 +1777,13 @@
     </row>
     <row r="13" spans="1:6">
       <c r="A13" t="s">
+        <v>100</v>
+      </c>
+      <c r="B13" t="s">
         <v>101</v>
       </c>
-      <c r="B13" t="s">
-        <v>102</v>
-      </c>
       <c r="C13" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="D13">
         <f>D12-Raw_Data!D10</f>
@@ -1722,13 +1799,13 @@
     </row>
     <row r="14" spans="1:6">
       <c r="A14" t="s">
+        <v>102</v>
+      </c>
+      <c r="B14" t="s">
         <v>103</v>
       </c>
-      <c r="B14" t="s">
+      <c r="C14" t="s">
         <v>104</v>
-      </c>
-      <c r="C14" t="s">
-        <v>105</v>
       </c>
       <c r="D14" s="17">
         <f>D13/D6</f>
@@ -1744,13 +1821,13 @@
     </row>
     <row r="15" spans="1:6" ht="28.8">
       <c r="A15" t="s">
+        <v>105</v>
+      </c>
+      <c r="B15" s="12" t="s">
         <v>106</v>
       </c>
-      <c r="B15" s="12" t="s">
+      <c r="C15" t="s">
         <v>107</v>
-      </c>
-      <c r="C15" t="s">
-        <v>108</v>
       </c>
       <c r="D15" s="18">
         <f>Raw_Data!D14/Raw_Data!D2*365</f>
@@ -1766,13 +1843,13 @@
     </row>
     <row r="16" spans="1:6" ht="28.8">
       <c r="A16" t="s">
+        <v>108</v>
+      </c>
+      <c r="B16" s="12" t="s">
         <v>109</v>
       </c>
-      <c r="B16" s="12" t="s">
-        <v>110</v>
-      </c>
       <c r="C16" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="D16">
         <f>Raw_Data!D3*(1-$D$2)</f>
@@ -1789,13 +1866,13 @@
     </row>
     <row r="17" spans="1:6" ht="28.8">
       <c r="A17" t="s">
+        <v>110</v>
+      </c>
+      <c r="B17" s="12" t="s">
         <v>111</v>
       </c>
-      <c r="B17" s="12" t="s">
-        <v>112</v>
-      </c>
       <c r="C17" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="D17">
         <f>D12+Raw_Data!D13-Raw_Data!D10</f>
@@ -1811,13 +1888,13 @@
     </row>
     <row r="18" spans="1:6" ht="28.8">
       <c r="A18" t="s">
+        <v>112</v>
+      </c>
+      <c r="B18" s="12" t="s">
         <v>113</v>
       </c>
-      <c r="B18" s="12" t="s">
-        <v>114</v>
-      </c>
       <c r="C18" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="D18" s="15">
         <f>D16/AVERAGE(D17:E17)</f>
@@ -1832,13 +1909,13 @@
     </row>
     <row r="19" spans="1:6" ht="28.8">
       <c r="A19" t="s">
+        <v>114</v>
+      </c>
+      <c r="B19" s="12" t="s">
         <v>115</v>
       </c>
-      <c r="B19" s="12" t="s">
-        <v>116</v>
-      </c>
       <c r="C19" s="19" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="D19" s="15">
         <f>D16/AVERAGE(D17-Raw_Data!D15,E17-Raw_Data!E15)</f>
@@ -1851,20 +1928,38 @@
         <v>62</v>
       </c>
     </row>
+    <row r="20" spans="1:6" ht="28.8">
+      <c r="A20" t="s">
+        <v>150</v>
+      </c>
+      <c r="B20" s="12" t="s">
+        <v>151</v>
+      </c>
+      <c r="C20" t="s">
+        <v>89</v>
+      </c>
+      <c r="D20" s="15">
+        <f>(Raw_Data!D2/Raw_Data!G2)^(1/3)-1</f>
+        <v>1.7466606469289658E-2</v>
+      </c>
+      <c r="E20" t="s">
+        <v>62</v>
+      </c>
+    </row>
     <row r="21" spans="1:6">
       <c r="A21" s="1" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="22" spans="1:6">
       <c r="A22" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="B22" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="C22" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="D22" s="20">
         <v>20.350000000000001</v>
@@ -1872,13 +1967,13 @@
     </row>
     <row r="23" spans="1:6">
       <c r="A23" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="B23" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="C23" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="D23" s="22">
         <f>D22*Raw_Data!D5</f>
@@ -1887,13 +1982,13 @@
     </row>
     <row r="24" spans="1:6">
       <c r="A24" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="B24" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="C24" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="D24" s="22">
         <f>D23+D13</f>
@@ -1902,13 +1997,13 @@
     </row>
     <row r="25" spans="1:6">
       <c r="A25" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="B25" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C25" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="D25" s="21">
         <f>D24/D6</f>
@@ -1917,13 +2012,13 @@
     </row>
     <row r="26" spans="1:6" ht="57.6">
       <c r="A26" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="B26" s="12" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="C26" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="D26" s="20">
         <v>866000</v>
@@ -1931,13 +2026,13 @@
     </row>
     <row r="27" spans="1:6" ht="28.8">
       <c r="A27" t="s">
+        <v>125</v>
+      </c>
+      <c r="B27" s="12" t="s">
         <v>126</v>
       </c>
-      <c r="B27" s="12" t="s">
-        <v>127</v>
-      </c>
       <c r="C27" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="D27" s="17">
         <f>D26/D6</f>
@@ -1962,27 +2057,27 @@
   <sheetData>
     <row r="1" spans="1:6">
       <c r="A1" s="1" t="s">
+        <v>130</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>131</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>132</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>133</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>134</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>135</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>136</v>
       </c>
     </row>
     <row r="2" spans="1:6">
       <c r="A2" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="B2" s="23">
         <v>250000</v>
@@ -2001,7 +2096,7 @@
     </row>
     <row r="3" spans="1:6">
       <c r="A3" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="B3" s="23">
         <v>40000</v>
@@ -2020,10 +2115,11 @@
     </row>
     <row r="4" spans="1:6">
       <c r="A4" t="s">
-        <v>91</v>
+        <v>152</v>
       </c>
       <c r="B4" s="24">
-        <v>0.05</v>
+        <f>Calculations!D20</f>
+        <v>1.7466606469289658E-2</v>
       </c>
       <c r="C4" s="23"/>
       <c r="D4" s="15">
@@ -2034,13 +2130,13 @@
         <f t="shared" si="0"/>
         <v>FAIL</v>
       </c>
-      <c r="F4" s="25" t="s">
-        <v>142</v>
+      <c r="F4" t="s">
+        <v>153</v>
       </c>
     </row>
     <row r="5" spans="1:6">
       <c r="A5" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B5" s="24">
         <v>0.12</v>
@@ -2055,12 +2151,12 @@
         <v>FAIL</v>
       </c>
       <c r="F5" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
     </row>
     <row r="6" spans="1:6">
       <c r="A6" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="B6" s="24">
         <v>0.7</v>
@@ -2075,12 +2171,12 @@
         <v>FAIL</v>
       </c>
       <c r="F6" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
     </row>
     <row r="7" spans="1:6">
       <c r="A7" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="B7" s="23"/>
       <c r="C7" s="24">
@@ -2095,12 +2191,12 @@
         <v>FAIL</v>
       </c>
       <c r="F7" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
     </row>
     <row r="8" spans="1:6">
       <c r="A8" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="B8" s="23"/>
       <c r="C8" s="23">
@@ -2115,12 +2211,12 @@
         <v>PASS</v>
       </c>
       <c r="F8" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
     </row>
     <row r="9" spans="1:6">
       <c r="A9" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="B9" s="23"/>
       <c r="C9" s="23">
@@ -2135,12 +2231,12 @@
         <v>FAIL</v>
       </c>
       <c r="F9" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
     </row>
     <row r="11" spans="1:6">
       <c r="A11" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="E11" t="str">
         <f>COUNTIF(E2:E9,"PASS")&amp;" of 8"</f>

</xml_diff>

<commit_message>
Add QuinStreet LBO model; max price analysis shows deal not actionable at market
</commit_message>
<xml_diff>
--- a/excel/mistras_answer_key.xlsx
+++ b/excel/mistras_answer_key.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rithu\Projects\pe-deal-screening-engine\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CABE7593-68AD-4830-BBFB-1A254C4CACDE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D252F2EE-896A-4F69-A6BC-CED3D54026E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{86B3820A-0EC3-49A7-AC89-EEF969BD1741}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{86B3820A-0EC3-49A7-AC89-EEF969BD1741}"/>
   </bookViews>
   <sheets>
     <sheet name="Source" sheetId="1" r:id="rId1"/>
@@ -2118,13 +2118,12 @@
         <v>152</v>
       </c>
       <c r="B4" s="24">
+        <v>0.05</v>
+      </c>
+      <c r="C4" s="23"/>
+      <c r="D4" s="15">
         <f>Calculations!D20</f>
         <v>1.7466606469289658E-2</v>
-      </c>
-      <c r="C4" s="23"/>
-      <c r="D4" s="15">
-        <f>Calculations!D8</f>
-        <v>-7.6969464393399356E-3</v>
       </c>
       <c r="E4" t="str">
         <f t="shared" si="0"/>

</xml_diff>